<commit_message>
Archive Spring 2026 semester: commit all end-of-semester files
Adds all previously untracked content (coding demos, exams, grading
outputs, notes, problems, scripts, meta) and final grading changes.
Full semester state preserved before archiving.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/src/grading/course/outputs/202610_Economics_1001_01_Filled.xlsx
+++ b/src/grading/course/outputs/202610_Economics_1001_01_Filled.xlsx
@@ -1169,7 +1169,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>A-</t>
+          <t>A</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
@@ -1686,7 +1686,7 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>B+</t>
+          <t>A-</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
@@ -2579,7 +2579,7 @@
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>B-</t>
+          <t>B</t>
         </is>
       </c>
       <c r="M47" t="inlineStr">
@@ -7462,7 +7462,7 @@
       </c>
       <c r="H151" t="inlineStr">
         <is>
-          <t>B+</t>
+          <t>A-</t>
         </is>
       </c>
       <c r="M151" t="inlineStr">
@@ -8308,7 +8308,7 @@
       </c>
       <c r="H169" t="inlineStr">
         <is>
-          <t>A-</t>
+          <t>A</t>
         </is>
       </c>
       <c r="M169" t="inlineStr">
@@ -11081,7 +11081,7 @@
       </c>
       <c r="H228" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>B+</t>
         </is>
       </c>
       <c r="M228" t="inlineStr">

</xml_diff>